<commit_message>
Adding and refactoring some of files
</commit_message>
<xml_diff>
--- a/public/medical_codes.xlsx
+++ b/public/medical_codes.xlsx
@@ -1,76 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UI-Based\mediclaim-ai\mediclaim-ai\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861A995A-6D0D-453C-B5BF-C429B9266CD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7DEB1F-37D1-4A72-A559-DA3219F23D69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Extracted Codes Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="CPT Codes" sheetId="2" r:id="rId2"/>
-    <sheet name="NDC Medication Codes" sheetId="3" r:id="rId3"/>
-    <sheet name="Related Codes" sheetId="4" r:id="rId4"/>
-    <sheet name="Diagnosis Codes" sheetId="5" r:id="rId5"/>
+    <sheet name="CPT Codes" sheetId="2" r:id="rId1"/>
+    <sheet name="NDC Medication Codes" sheetId="3" r:id="rId2"/>
+    <sheet name="Related Codes" sheetId="4" r:id="rId3"/>
+    <sheet name="Diagnosis Codes" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="207">
   <si>
     <t>Code Type</t>
   </si>
   <si>
-    <t>Code</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
-    <t>Amount</t>
-  </si>
-  <si>
     <t>Patient</t>
   </si>
   <si>
-    <t>Date of Service</t>
-  </si>
-  <si>
-    <t>Insurance</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>CPT</t>
-  </si>
-  <si>
     <t>99213</t>
   </si>
   <si>
     <t>Office/outpatient visit - established patient, low complexity</t>
   </si>
   <si>
-    <t>$120.00</t>
-  </si>
-  <si>
     <t>Cici George</t>
   </si>
   <si>
-    <t>11/20/2024</t>
-  </si>
-  <si>
-    <t>Blue Cross PPO</t>
-  </si>
-  <si>
     <t>E/M</t>
   </si>
   <si>
@@ -80,9 +52,6 @@
     <t>Rapid influenza test</t>
   </si>
   <si>
-    <t>$35.00</t>
-  </si>
-  <si>
     <t>Lab/Pathology</t>
   </si>
   <si>
@@ -92,39 +61,21 @@
     <t>COVID-19 antigen test</t>
   </si>
   <si>
-    <t>$25.00</t>
-  </si>
-  <si>
-    <t>NDC</t>
-  </si>
-  <si>
     <t>0069-0239-68</t>
   </si>
   <si>
-    <t>Amoxicillin 500mg (30 tablets)</t>
-  </si>
-  <si>
     <t>$45.00</t>
   </si>
   <si>
-    <t>Medication</t>
-  </si>
-  <si>
     <t>0093-7643-01</t>
   </si>
   <si>
-    <t>Ibuprofen 600mg (60 tablets)</t>
-  </si>
-  <si>
     <t>$18.00</t>
   </si>
   <si>
     <t>0088-7666-32</t>
   </si>
   <si>
-    <t>Acetaminophen 500mg (30 tablets)</t>
-  </si>
-  <si>
     <t>$12.00</t>
   </si>
   <si>
@@ -134,9 +85,6 @@
     <t>Office/outpatient visit - established patient, moderate complexity</t>
   </si>
   <si>
-    <t>$135.00</t>
-  </si>
-  <si>
     <t>Jill Francis</t>
   </si>
   <si>
@@ -146,9 +94,6 @@
     <t>Pertussis (whooping cough) PCR test</t>
   </si>
   <si>
-    <t>$95.00</t>
-  </si>
-  <si>
     <t>99000</t>
   </si>
   <si>
@@ -164,48 +109,27 @@
     <t>Chest X-ray, 2 views</t>
   </si>
   <si>
-    <t>$80.00</t>
-  </si>
-  <si>
     <t>Radiology</t>
   </si>
   <si>
     <t>0002-3106-50</t>
   </si>
   <si>
-    <t>Azithromycin 200mg/5ml suspension</t>
-  </si>
-  <si>
     <t>$65.00</t>
   </si>
   <si>
     <t>0378-9130-01</t>
   </si>
   <si>
-    <t>Benzonatate 100mg capsules</t>
-  </si>
-  <si>
     <t>$28.00</t>
   </si>
   <si>
     <t>0088-1658-32</t>
   </si>
   <si>
-    <t>Diphenhydramine 12.5mg syrup</t>
-  </si>
-  <si>
     <t>$16.00</t>
   </si>
   <si>
-    <t>$175.00</t>
-  </si>
-  <si>
-    <t>Mary Johnson</t>
-  </si>
-  <si>
-    <t>Aetna PPO</t>
-  </si>
-  <si>
     <t>93000</t>
   </si>
   <si>
@@ -216,9 +140,6 @@
   </si>
   <si>
     <t>36415</t>
-  </si>
-  <si>
-    <t>Venipuncture, single puncture</t>
   </si>
   <si>
     <t>CPT Code</t>
@@ -1097,468 +1018,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="15" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1573,42 +1032,42 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>70</v>
+        <v>44</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3">
         <v>0.97</v>
@@ -1620,24 +1079,24 @@
         <v>110</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="D3" s="3">
         <v>1.5</v>
@@ -1649,24 +1108,24 @@
         <v>220</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D4" s="3">
         <v>0.26</v>
@@ -1678,24 +1137,24 @@
         <v>65</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D5" s="3">
         <v>0.24</v>
@@ -1707,24 +1166,24 @@
         <v>50</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3">
         <v>0.55000000000000004</v>
@@ -1736,24 +1195,24 @@
         <v>120</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>79</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="D7" s="3">
         <v>0.15</v>
@@ -1765,24 +1224,24 @@
         <v>35</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="D8" s="3">
         <v>0.45</v>
@@ -1794,24 +1253,24 @@
         <v>150</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>61</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>62</v>
+        <v>37</v>
       </c>
       <c r="D9" s="3">
         <v>0.14000000000000001</v>
@@ -1823,24 +1282,24 @@
         <v>75</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>83</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3">
         <v>0.04</v>
@@ -1852,13 +1311,13 @@
         <v>30</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1866,7 +1325,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1884,205 +1343,205 @@
   <sheetData>
     <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>97</v>
+        <v>71</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>103</v>
+        <v>77</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>29</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>105</v>
+        <v>79</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>107</v>
+        <v>81</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>108</v>
+        <v>82</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>109</v>
+        <v>83</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>110</v>
+        <v>84</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>112</v>
+        <v>86</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>114</v>
+        <v>88</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>115</v>
+        <v>89</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>116</v>
+        <v>90</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -2090,7 +1549,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2105,42 +1564,42 @@
   <sheetData>
     <row r="1" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>118</v>
+        <v>92</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>119</v>
+        <v>93</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>120</v>
+        <v>94</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>121</v>
+        <v>95</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>122</v>
+        <v>96</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>123</v>
+        <v>97</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>124</v>
+        <v>98</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>125</v>
+        <v>99</v>
       </c>
       <c r="F2" s="3">
         <v>60</v>
@@ -2151,19 +1610,19 @@
     </row>
     <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>126</v>
+        <v>100</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>127</v>
+        <v>101</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>129</v>
+        <v>103</v>
       </c>
       <c r="F3" s="3">
         <v>60</v>
@@ -2174,19 +1633,19 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>130</v>
+        <v>104</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>132</v>
+        <v>106</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>133</v>
+        <v>107</v>
       </c>
       <c r="F4" s="3">
         <v>350</v>
@@ -2197,19 +1656,19 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>135</v>
+        <v>109</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F5" s="3">
         <v>20</v>
@@ -2220,19 +1679,19 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>138</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>113</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>136</v>
+        <v>110</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F6" s="3">
         <v>20</v>
@@ -2243,19 +1702,19 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>140</v>
+        <v>114</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>141</v>
+        <v>115</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>142</v>
+        <v>116</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="F7" s="3">
         <v>20</v>
@@ -2266,19 +1725,19 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>144</v>
+        <v>118</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>145</v>
+        <v>119</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>146</v>
+        <v>120</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F8" s="3">
         <v>30</v>
@@ -2289,19 +1748,19 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>147</v>
+        <v>121</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>148</v>
+        <v>122</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>149</v>
+        <v>123</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F9" s="3">
         <v>50</v>
@@ -2312,19 +1771,19 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>150</v>
+        <v>124</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>151</v>
+        <v>125</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>152</v>
+        <v>126</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="F10" s="3">
         <v>40</v>
@@ -2335,19 +1794,19 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>154</v>
+        <v>128</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>156</v>
+        <v>130</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>153</v>
+        <v>127</v>
       </c>
       <c r="F11" s="3">
         <v>80</v>
@@ -2358,19 +1817,19 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>157</v>
+        <v>131</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>158</v>
+        <v>132</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>159</v>
+        <v>133</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>160</v>
+        <v>134</v>
       </c>
       <c r="F12" s="3">
         <v>30</v>
@@ -2381,19 +1840,19 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>60</v>
+        <v>35</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>161</v>
+        <v>135</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>163</v>
+        <v>137</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>143</v>
+        <v>117</v>
       </c>
       <c r="F13" s="3">
         <v>35</v>
@@ -2404,19 +1863,19 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>164</v>
+        <v>138</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>165</v>
+        <v>139</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>166</v>
+        <v>140</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>167</v>
+        <v>141</v>
       </c>
       <c r="F14" s="3">
         <v>8</v>
@@ -2427,19 +1886,19 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>168</v>
+        <v>142</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>169</v>
+        <v>143</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="F15" s="3">
         <v>90</v>
@@ -2450,19 +1909,19 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>146</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>173</v>
+        <v>147</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>170</v>
+        <v>144</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>171</v>
+        <v>145</v>
       </c>
       <c r="F16" s="3">
         <v>130</v>
@@ -2476,7 +1935,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2491,222 +1950,222 @@
   <sheetData>
     <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>174</v>
+        <v>148</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>175</v>
+        <v>149</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>176</v>
+        <v>150</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>177</v>
+        <v>151</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>178</v>
+        <v>152</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>179</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>181</v>
+        <v>155</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>186</v>
+        <v>160</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>187</v>
+        <v>161</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>188</v>
+        <v>162</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>189</v>
+        <v>163</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>191</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>192</v>
+        <v>166</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>193</v>
+        <v>167</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>194</v>
+        <v>168</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>195</v>
+        <v>169</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>197</v>
+        <v>171</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>198</v>
+        <v>172</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>199</v>
+        <v>173</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>200</v>
+        <v>174</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>201</v>
+        <v>175</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>202</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>203</v>
+        <v>177</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>204</v>
+        <v>178</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>205</v>
+        <v>179</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>206</v>
+        <v>180</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>207</v>
+        <v>181</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>209</v>
+        <v>183</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>210</v>
+        <v>184</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>214</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>215</v>
+        <v>189</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>211</v>
+        <v>185</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>217</v>
+        <v>191</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>220</v>
+        <v>194</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>222</v>
+        <v>196</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>223</v>
+        <v>197</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>225</v>
+        <v>199</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>226</v>
+        <v>200</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>190</v>
+        <v>164</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>196</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>227</v>
+        <v>201</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>228</v>
+        <v>202</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>229</v>
+        <v>203</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>230</v>
+        <v>204</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>231</v>
+        <v>205</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>232</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>